<commit_message>
changed pin header to a smaller one and removed USB secondary power supply
</commit_message>
<xml_diff>
--- a/karca_v2_testing.xlsx
+++ b/karca_v2_testing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Deepak\Documents\kARCA_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71C1337C-09EA-40E0-BD80-C1B39C8D4D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C604A2-999C-45CC-8031-54C058CCF32F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1790" yWindow="1830" windowWidth="18150" windowHeight="7270" xr2:uid="{9DD3C288-D188-4B64-8C3D-0D87CD283653}"/>
+    <workbookView xWindow="1140" yWindow="120" windowWidth="18150" windowHeight="7270" xr2:uid="{9DD3C288-D188-4B64-8C3D-0D87CD283653}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="69">
   <si>
     <t>Current</t>
   </si>
@@ -234,6 +234,15 @@
   </si>
   <si>
     <t>pt is having issues</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>i</t>
   </si>
 </sst>
 </file>
@@ -641,7 +650,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B0411DD-F165-47C3-8FE1-CF4160B1F7AD}">
-  <dimension ref="A1:R58"/>
+  <dimension ref="A1:S58"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.35">
@@ -1211,7 +1220,7 @@
         <v>0.52500000000000002</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
       <c r="K33">
         <f>(50/150)*12</f>
         <v>4</v>
@@ -1221,7 +1230,7 @@
         <v>10.004999999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A34" s="8" t="s">
         <v>44</v>
       </c>
@@ -1229,7 +1238,7 @@
       <c r="C34" s="8"/>
       <c r="D34" s="8"/>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>45</v>
       </c>
@@ -1243,7 +1252,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>48</v>
       </c>
@@ -1261,7 +1270,7 @@
         <v>0.29145507812499999</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>49</v>
       </c>
@@ -1279,7 +1288,7 @@
         <v>9.5663818359375004</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>50</v>
       </c>
@@ -1298,7 +1307,7 @@
         <v>1.028125</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A40" s="8" t="s">
         <v>53</v>
       </c>
@@ -1306,7 +1315,7 @@
       <c r="C40" s="8"/>
       <c r="D40" s="8"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -1320,7 +1329,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A42" s="8" t="s">
         <v>54</v>
       </c>
@@ -1338,7 +1347,7 @@
         <v>0.5794677734375</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A43" s="8"/>
       <c r="B43">
         <v>1</v>
@@ -1351,7 +1360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A44" s="8"/>
       <c r="B44">
         <v>1.67</v>
@@ -1367,7 +1376,7 @@
         <v>1.6902099609375001</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A45" s="8"/>
       <c r="B45">
         <v>2</v>
@@ -1377,7 +1386,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A46" s="8"/>
       <c r="B46">
         <v>2.7</v>
@@ -1392,16 +1401,38 @@
         <f t="shared" si="8"/>
         <v>2.7699707031250003</v>
       </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="O46" t="s">
+        <v>67</v>
+      </c>
+      <c r="P46" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="O47">
+        <v>0</v>
+      </c>
+      <c r="P47">
+        <f>O47/200</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A48" s="8" t="s">
         <v>56</v>
       </c>
       <c r="B48" s="8"/>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="O48">
+        <v>0.5</v>
+      </c>
+      <c r="P48">
+        <f t="shared" ref="P48:P53" si="9">O48/200</f>
+        <v>2.5000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>45</v>
       </c>
@@ -1414,8 +1445,15 @@
       <c r="D49" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="O49">
+        <v>1</v>
+      </c>
+      <c r="P49">
+        <f t="shared" si="9"/>
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>57</v>
       </c>
@@ -1437,8 +1475,15 @@
         <f>2.5/0.34</f>
         <v>7.3529411764705879</v>
       </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="O50">
+        <v>1.5</v>
+      </c>
+      <c r="P50">
+        <f t="shared" si="9"/>
+        <v>7.4999999999999997E-3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>58</v>
       </c>
@@ -1446,15 +1491,22 @@
         <v>0</v>
       </c>
       <c r="D51">
-        <f t="shared" ref="D51:D52" si="9">G51/(200*0.01)</f>
+        <f t="shared" ref="D51:D52" si="10">G51/(200*0.01)</f>
         <v>0</v>
       </c>
       <c r="G51">
-        <f t="shared" ref="G51:G54" si="10">(C51*4.7)/4096</f>
+        <f t="shared" ref="G51:G54" si="11">(C51*4.7)/4096</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="O51">
+        <v>2</v>
+      </c>
+      <c r="P51">
+        <f t="shared" si="9"/>
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="52" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>59</v>
       </c>
@@ -1465,15 +1517,22 @@
         <v>886</v>
       </c>
       <c r="D52">
+        <f t="shared" si="10"/>
+        <v>0.50832519531249998</v>
+      </c>
+      <c r="G52">
+        <f t="shared" si="11"/>
+        <v>1.016650390625</v>
+      </c>
+      <c r="O52">
+        <v>2.5</v>
+      </c>
+      <c r="P52">
         <f t="shared" si="9"/>
-        <v>0.50832519531249998</v>
-      </c>
-      <c r="G52">
-        <f t="shared" si="10"/>
-        <v>1.016650390625</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
+        <v>1.2500000000000001E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>60</v>
       </c>
@@ -1484,11 +1543,18 @@
         <v>882</v>
       </c>
       <c r="G53">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>1.0120605468750001</v>
       </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="O53">
+        <v>3</v>
+      </c>
+      <c r="P53">
+        <f t="shared" si="9"/>
+        <v>1.4999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>61</v>
       </c>
@@ -1499,26 +1565,29 @@
         <v>4085</v>
       </c>
       <c r="G54">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>4.6873779296875</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="S56" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="57" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B58" t="s">
         <v>65</v>
       </c>

</xml_diff>